<commit_message>
Add center transfers, analytics, and admin center management features
Introduces inter-center stock transfers (routes/transfers.js, AdminTransfers
page), per-center analytics dashboard, MyCenter admin view, and self-service
center registration landing page. Adds supporting scripts (reset-fresh-launch,
updateGopalanInventory, migrate_users), backend tests, and consolidates
duplicate inventory-sync logic into backend/scripts/legacy with deprecated
stubs left in place per CLEANUP.md. Also adds training/reference docs
(cheat sheets, user manuals, training packs, deployment guide) and syncs
current center data snapshots.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/jp_nagar/jp_nagar_logs.xlsx
+++ b/backend/data/jp_nagar/jp_nagar_logs.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2045" uniqueCount="213">
   <si>
     <t>Timestamp</t>
   </si>
@@ -479,6 +479,177 @@
   </si>
   <si>
     <t>super_admin</t>
+  </si>
+  <si>
+    <t>jp_nagar_student1</t>
+  </si>
+  <si>
+    <t>jp_nagar_admin</t>
+  </si>
+  <si>
+    <t>Order CIMS-MNN6FTP1: 2 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>Order CIMS-MNN8GCS4: 2 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>Order CIMS-MNN8KP6J: 1 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>Order CIMS-MNN8MNZJ: 1 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>Order CIMS-MNN8Z5ST: 1 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>CIMS-MNN8Z5ST -&gt; Approved</t>
+  </si>
+  <si>
+    <t>CIMS-MNN8MNZJ -&gt; Rejected</t>
+  </si>
+  <si>
+    <t>Updated user: jp_nagar_admin</t>
+  </si>
+  <si>
+    <t>CIMS-MNN8KP6J -&gt; Rejected</t>
+  </si>
+  <si>
+    <t>CIMS-MNN8GCS4 -&gt; Rejected</t>
+  </si>
+  <si>
+    <t>CIMS-MNN6FTP1 -&gt; Rejected</t>
+  </si>
+  <si>
+    <t>CIMS-MNN8Z5ST marked for return</t>
+  </si>
+  <si>
+    <t>CIMS-MNN8Z5ST -&gt; Returned</t>
+  </si>
+  <si>
+    <t>Order CIMS-MNOAT2L6: 1 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>CIMS-MNOAT2L6 -&gt; Approved</t>
+  </si>
+  <si>
+    <t>CIMS-MNOAT2L6 marked for return</t>
+  </si>
+  <si>
+    <t>CIMS-MNOAT2L6 -&gt; Returned</t>
+  </si>
+  <si>
+    <t>Added: Power Bank 10000 mAh</t>
+  </si>
+  <si>
+    <t>Order CIMS-MNOBJ1FA: 2 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>CIMS-MNOBJ1FA -&gt; Approved</t>
+  </si>
+  <si>
+    <t>Order CIMS-MNR4L8JK: 3 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>CIMS-MNR4L8JK -&gt; Approved</t>
+  </si>
+  <si>
+    <t>Order CIMS-MNR4S171: 1 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>CIMS-MNR4S171 -&gt; Approved</t>
+  </si>
+  <si>
+    <t>CIMS-MNR4S171 marked for return</t>
+  </si>
+  <si>
+    <t>CIMS-MNR4L8JK marked for return</t>
+  </si>
+  <si>
+    <t>CIMS-MNOBJ1FA marked for return</t>
+  </si>
+  <si>
+    <t>CIMS-MNR4S171 -&gt; Returned</t>
+  </si>
+  <si>
+    <t>CIMS-MNR4L8JK -&gt; Returned</t>
+  </si>
+  <si>
+    <t>CIMS-MNOBJ1FA -&gt; Returned</t>
+  </si>
+  <si>
+    <t>TRANSFER_REQUEST</t>
+  </si>
+  <si>
+    <t>Requested 1 components (Transfer 84cd6f1e-86d8-4ee2-a380-2691a7f165ac)</t>
+  </si>
+  <si>
+    <t>TRANSFER_APPROVED</t>
+  </si>
+  <si>
+    <t>Transfer 84cd6f1e-86d8-4ee2-a380-2691a7f165ac approved (supplied by yelahanka)</t>
+  </si>
+  <si>
+    <t>TRANSFER_RETURN_REQUESTED</t>
+  </si>
+  <si>
+    <t>Return requested for 84cd6f1e-86d8-4ee2-a380-2691a7f165ac</t>
+  </si>
+  <si>
+    <t>TRANSFER_RETURNED</t>
+  </si>
+  <si>
+    <t>Transfer 84cd6f1e-86d8-4ee2-a380-2691a7f165ac returned to yelahanka</t>
+  </si>
+  <si>
+    <t>guru</t>
+  </si>
+  <si>
+    <t>Updated user: guru</t>
+  </si>
+  <si>
+    <t>Deleted user: b19a3d02-0658-4b8c-bbce-bdb1d99a02b8</t>
+  </si>
+  <si>
+    <t>Order CIMS-MNTZL31E: 3 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>CIMS-MNTZL31E -&gt; Approved</t>
+  </si>
+  <si>
+    <t>CIMS-MNTZL31E marked for return</t>
+  </si>
+  <si>
+    <t>CIMS-MNTZL31E -&gt; Partially Returned</t>
+  </si>
+  <si>
+    <t>Updated user: superadmin</t>
+  </si>
+  <si>
+    <t>dhavalya</t>
+  </si>
+  <si>
+    <t>Pragathi</t>
+  </si>
+  <si>
+    <t>Updated user: dhavalya</t>
+  </si>
+  <si>
+    <t>Updated user: Pragathi</t>
+  </si>
+  <si>
+    <t>Updated ID: b3e9f1d7-ca6b-44a9-9e03-11ef1b3ccf10</t>
+  </si>
+  <si>
+    <t>Order CIMS-MP7YCN2Z: 6 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>CIMS-MP7YCN2Z -&gt; Approved</t>
+  </si>
+  <si>
+    <t>Order CIMS-MP7Z6CV3: 7 component type(s) reserved</t>
+  </si>
+  <si>
+    <t>CIMS-MP7Z6CV3 -&gt; Approved</t>
   </si>
 </sst>
 </file>
@@ -904,7 +1075,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G259"/>
+  <dimension ref="A1:G424"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -5373,6 +5544,3801 @@
         <v>9</v>
       </c>
     </row>
+    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A260" s="2">
+        <v>46118.48652881944</v>
+      </c>
+      <c r="B260" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C260" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D260" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E260" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F260" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G260" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A261" s="4">
+        <v>46118.4916265162</v>
+      </c>
+      <c r="B261" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C261" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D261" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E261" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F261" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G261" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A262" s="2">
+        <v>46118.49275520833</v>
+      </c>
+      <c r="B262" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C262" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D262" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E262" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F262" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G262" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A263" s="4">
+        <v>46118.49578246528</v>
+      </c>
+      <c r="B263" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C263" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D263" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E263" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F263" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G263" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A264" s="2">
+        <v>46118.501519513884</v>
+      </c>
+      <c r="B264" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C264" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D264" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E264" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F264" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G264" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A265" s="4">
+        <v>46118.50241806713</v>
+      </c>
+      <c r="B265" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C265" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D265" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E265" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F265" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G265" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A266" s="2">
+        <v>46118.50370385416</v>
+      </c>
+      <c r="B266" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C266" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D266" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E266" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F266" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G266" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A267" s="4">
+        <v>46118.50829787037</v>
+      </c>
+      <c r="B267" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C267" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D267" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="E267" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F267" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G267" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A268" s="2">
+        <v>46118.522246030094</v>
+      </c>
+      <c r="B268" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C268" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D268" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E268" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F268" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G268" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A269" s="4">
+        <v>46118.52301133102</v>
+      </c>
+      <c r="B269" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C269" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D269" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E269" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F269" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G269" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A270" s="2">
+        <v>46118.524819108796</v>
+      </c>
+      <c r="B270" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C270" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D270" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E270" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F270" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G270" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A271" s="4">
+        <v>46118.52621844907</v>
+      </c>
+      <c r="B271" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C271" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D271" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E271" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F271" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G271" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A272" s="2">
+        <v>46118.52642758102</v>
+      </c>
+      <c r="B272" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C272" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D272" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E272" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F272" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G272" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A273" s="4">
+        <v>46118.526460023146</v>
+      </c>
+      <c r="B273" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C273" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D273" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E273" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F273" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G273" s="5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A274" s="2">
+        <v>46118.5264819213</v>
+      </c>
+      <c r="B274" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C274" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D274" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E274" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F274" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G274" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A275" s="4">
+        <v>46118.527104050925</v>
+      </c>
+      <c r="B275" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C275" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D275" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E275" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F275" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G275" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="276" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A276" s="2">
+        <v>46118.527105625</v>
+      </c>
+      <c r="B276" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C276" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D276" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E276" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F276" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G276" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A277" s="4">
+        <v>46118.5659329051</v>
+      </c>
+      <c r="B277" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C277" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D277" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E277" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F277" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G277" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A278" s="2">
+        <v>46118.56626936342</v>
+      </c>
+      <c r="B278" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C278" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D278" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E278" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F278" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G278" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A279" s="4">
+        <v>46118.56627202546</v>
+      </c>
+      <c r="B279" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C279" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D279" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E279" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F279" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G279" s="5" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A280" s="2">
+        <v>46118.56861420139</v>
+      </c>
+      <c r="B280" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C280" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D280" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E280" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F280" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G280" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A281" s="4">
+        <v>46118.56861834491</v>
+      </c>
+      <c r="B281" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C281" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D281" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E281" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F281" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G281" s="5" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A282" s="2">
+        <v>46118.569677708336</v>
+      </c>
+      <c r="B282" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C282" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D282" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E282" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F282" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G282" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A283" s="4">
+        <v>46118.569680092594</v>
+      </c>
+      <c r="B283" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C283" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D283" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E283" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F283" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G283" s="5" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A284" s="2">
+        <v>46118.5762296412</v>
+      </c>
+      <c r="B284" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C284" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D284" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E284" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F284" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G284" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A285" s="4">
+        <v>46118.576425127314</v>
+      </c>
+      <c r="B285" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C285" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D285" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E285" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F285" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G285" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A286" s="2">
+        <v>46118.57642725694</v>
+      </c>
+      <c r="B286" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C286" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D286" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E286" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F286" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G286" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A287" s="4">
+        <v>46118.57764552083</v>
+      </c>
+      <c r="B287" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C287" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D287" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E287" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F287" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G287" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A288" s="2">
+        <v>46118.57821466435</v>
+      </c>
+      <c r="B288" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C288" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D288" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E288" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F288" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G288" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A289" s="4">
+        <v>46118.6607096875</v>
+      </c>
+      <c r="B289" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C289" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D289" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E289" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F289" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G289" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="290" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A290" s="2">
+        <v>46118.66104798611</v>
+      </c>
+      <c r="B290" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C290" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D290" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E290" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F290" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G290" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A291" s="4">
+        <v>46118.661123252314</v>
+      </c>
+      <c r="B291" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C291" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D291" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E291" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F291" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G291" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A292" s="2">
+        <v>46119.187502719906</v>
+      </c>
+      <c r="B292" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C292" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D292" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E292" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F292" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G292" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A293" s="4">
+        <v>46119.1912887037</v>
+      </c>
+      <c r="B293" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C293" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D293" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E293" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F293" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G293" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A294" s="2">
+        <v>46119.19154670139</v>
+      </c>
+      <c r="B294" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C294" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D294" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E294" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F294" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G294" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A295" s="4">
+        <v>46119.192160798615</v>
+      </c>
+      <c r="B295" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C295" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D295" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E295" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F295" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G295" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A296" s="2">
+        <v>46119.19292180556</v>
+      </c>
+      <c r="B296" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C296" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D296" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E296" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F296" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G296" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A297" s="4">
+        <v>46119.19346434028</v>
+      </c>
+      <c r="B297" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C297" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D297" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E297" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F297" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G297" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A298" s="2">
+        <v>46119.19381600694</v>
+      </c>
+      <c r="B298" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C298" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D298" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E298" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F298" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G298" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A299" s="4">
+        <v>46119.19407798611</v>
+      </c>
+      <c r="B299" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C299" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D299" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E299" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F299" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G299" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A300" s="2">
+        <v>46119.19574283565</v>
+      </c>
+      <c r="B300" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C300" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D300" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E300" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F300" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G300" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="301" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A301" s="4">
+        <v>46119.197220092596</v>
+      </c>
+      <c r="B301" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C301" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D301" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E301" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F301" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G301" s="5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="302" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A302" s="2">
+        <v>46119.19726615741</v>
+      </c>
+      <c r="B302" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C302" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D302" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E302" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F302" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G302" s="3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="303" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A303" s="4">
+        <v>46119.19730238426</v>
+      </c>
+      <c r="B303" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C303" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D303" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E303" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F303" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G303" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="304" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A304" s="2">
+        <v>46119.19837491898</v>
+      </c>
+      <c r="B304" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C304" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D304" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E304" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F304" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G304" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A305" s="4">
+        <v>46119.1987037037</v>
+      </c>
+      <c r="B305" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C305" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D305" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E305" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F305" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G305" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="306" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A306" s="2">
+        <v>46119.19889576389</v>
+      </c>
+      <c r="B306" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C306" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D306" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E306" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F306" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G306" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="307" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A307" s="4">
+        <v>46119.19938553241</v>
+      </c>
+      <c r="B307" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C307" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D307" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E307" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F307" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G307" s="5" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="308" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A308" s="2">
+        <v>46119.205224398145</v>
+      </c>
+      <c r="B308" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C308" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D308" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E308" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F308" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G308" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="309" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A309" s="4">
+        <v>46119.26407208333</v>
+      </c>
+      <c r="B309" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C309" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D309" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E309" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F309" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G309" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="310" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A310" s="2">
+        <v>46119.27287615741</v>
+      </c>
+      <c r="B310" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C310" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D310" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E310" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F310" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G310" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="311" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A311" s="4">
+        <v>46119.31152859954</v>
+      </c>
+      <c r="B311" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C311" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D311" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E311" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F311" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G311" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="312" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A312" s="2">
+        <v>46119.31185697917</v>
+      </c>
+      <c r="B312" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C312" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D312" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E312" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F312" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G312" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="313" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A313" s="4">
+        <v>46119.31185914352</v>
+      </c>
+      <c r="B313" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C313" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D313" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E313" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F313" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G313" s="5" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="314" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A314" s="2">
+        <v>46119.31691871528</v>
+      </c>
+      <c r="B314" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C314" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D314" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E314" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F314" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G314" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="315" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A315" s="4">
+        <v>46119.31708449074</v>
+      </c>
+      <c r="B315" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C315" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D315" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E315" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F315" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G315" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="316" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A316" s="2">
+        <v>46119.31757185185</v>
+      </c>
+      <c r="B316" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C316" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D316" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E316" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F316" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G316" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="317" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A317" s="4">
+        <v>46119.31769899305</v>
+      </c>
+      <c r="B317" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C317" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D317" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E317" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F317" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G317" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="318" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A318" s="2">
+        <v>46119.317919305555</v>
+      </c>
+      <c r="B318" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C318" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D318" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E318" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F318" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G318" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="319" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A319" s="4">
+        <v>46119.32383122685</v>
+      </c>
+      <c r="B319" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C319" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D319" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E319" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F319" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G319" s="5" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="320" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A320" s="2">
+        <v>46119.32587731481</v>
+      </c>
+      <c r="B320" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C320" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D320" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E320" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F320" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G320" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="321" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A321" s="4">
+        <v>46119.325881655095</v>
+      </c>
+      <c r="B321" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C321" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D321" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E321" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F321" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G321" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="322" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A322" s="2">
+        <v>46119.326437696756</v>
+      </c>
+      <c r="B322" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C322" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D322" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E322" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F322" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G322" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="323" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A323" s="4">
+        <v>46120.25242125</v>
+      </c>
+      <c r="B323" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C323" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D323" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E323" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F323" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G323" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="324" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A324" s="2">
+        <v>46121.19784702546</v>
+      </c>
+      <c r="B324" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C324" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D324" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E324" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F324" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G324" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="325" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A325" s="4">
+        <v>46121.19807413194</v>
+      </c>
+      <c r="B325" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C325" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D325" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E325" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F325" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G325" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="326" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A326" s="2">
+        <v>46121.28911025463</v>
+      </c>
+      <c r="B326" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C326" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D326" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E326" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F326" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G326" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="327" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A327" s="4">
+        <v>46121.290018506945</v>
+      </c>
+      <c r="B327" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C327" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D327" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E327" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F327" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G327" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="328" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A328" s="2">
+        <v>46121.290505069446</v>
+      </c>
+      <c r="B328" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C328" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D328" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E328" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F328" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G328" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="329" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A329" s="4">
+        <v>46121.29050841436</v>
+      </c>
+      <c r="B329" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C329" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D329" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E329" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F329" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G329" s="5" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="330" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A330" s="2">
+        <v>46121.291099050926</v>
+      </c>
+      <c r="B330" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C330" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D330" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E330" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F330" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G330" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="331" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A331" s="4">
+        <v>46121.294176180556</v>
+      </c>
+      <c r="B331" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C331" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D331" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E331" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F331" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G331" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="332" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A332" s="2">
+        <v>46121.29417821759</v>
+      </c>
+      <c r="B332" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C332" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D332" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E332" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F332" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G332" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="333" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A333" s="4">
+        <v>46121.29451684028</v>
+      </c>
+      <c r="B333" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C333" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D333" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E333" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F333" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G333" s="5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="334" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A334" s="2">
+        <v>46121.29674809027</v>
+      </c>
+      <c r="B334" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C334" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D334" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E334" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F334" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G334" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="335" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A335" s="4">
+        <v>46121.29712618055</v>
+      </c>
+      <c r="B335" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C335" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D335" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E335" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F335" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G335" s="5" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="336" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A336" s="2">
+        <v>46121.29716209491</v>
+      </c>
+      <c r="B336" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C336" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D336" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E336" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F336" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G336" s="3" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="337" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A337" s="4">
+        <v>46121.29718612268</v>
+      </c>
+      <c r="B337" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C337" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D337" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E337" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F337" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G337" s="5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="338" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A338" s="2">
+        <v>46121.297368761574</v>
+      </c>
+      <c r="B338" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C338" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D338" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E338" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F338" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G338" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="339" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A339" s="4">
+        <v>46121.29745846065</v>
+      </c>
+      <c r="B339" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C339" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D339" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E339" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F339" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G339" s="5" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="340" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A340" s="2">
+        <v>46121.29754234954</v>
+      </c>
+      <c r="B340" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C340" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D340" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E340" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F340" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G340" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="341" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A341" s="4">
+        <v>46121.450030162036</v>
+      </c>
+      <c r="B341" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C341" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D341" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E341" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F341" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G341" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="342" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A342" s="2">
+        <v>46121.450217777776</v>
+      </c>
+      <c r="B342" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C342" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D342" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E342" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F342" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G342" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="343" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A343" s="4">
+        <v>46121.4508178588</v>
+      </c>
+      <c r="B343" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C343" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D343" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E343" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F343" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G343" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="344" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A344" s="2">
+        <v>46121.461347766206</v>
+      </c>
+      <c r="B344" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C344" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D344" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E344" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F344" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G344" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="345" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A345" s="4">
+        <v>46121.50028604167</v>
+      </c>
+      <c r="B345" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C345" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D345" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E345" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F345" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G345" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="346" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A346" s="2">
+        <v>46121.50893476851</v>
+      </c>
+      <c r="B346" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C346" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D346" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E346" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F346" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G346" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="347" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A347" s="4">
+        <v>46121.50905332176</v>
+      </c>
+      <c r="B347" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C347" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D347" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E347" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F347" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G347" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="348" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A348" s="2">
+        <v>46121.51532391204</v>
+      </c>
+      <c r="B348" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C348" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D348" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E348" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F348" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G348" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="349" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A349" s="4">
+        <v>46121.516089375</v>
+      </c>
+      <c r="B349" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C349" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D349" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E349" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F349" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G349" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="350" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A350" s="2">
+        <v>46121.52267003473</v>
+      </c>
+      <c r="B350" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C350" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D350" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E350" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F350" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G350" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="351" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A351" s="4">
+        <v>46121.52755359954</v>
+      </c>
+      <c r="B351" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C351" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D351" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E351" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F351" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G351" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="352" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A352" s="2">
+        <v>46122.21175630787</v>
+      </c>
+      <c r="B352" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C352" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D352" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E352" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F352" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G352" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="353" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A353" s="4">
+        <v>46122.31343759259</v>
+      </c>
+      <c r="B353" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C353" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D353" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E353" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F353" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G353" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="354" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A354" s="2">
+        <v>46122.317628530094</v>
+      </c>
+      <c r="B354" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C354" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D354" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E354" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F354" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G354" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="355" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A355" s="4">
+        <v>46122.31781807871</v>
+      </c>
+      <c r="B355" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C355" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D355" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E355" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F355" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G355" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="356" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A356" s="2">
+        <v>46122.331526793976</v>
+      </c>
+      <c r="B356" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C356" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D356" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E356" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F356" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G356" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="357" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A357" s="4">
+        <v>46122.33220517361</v>
+      </c>
+      <c r="B357" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C357" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D357" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E357" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F357" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G357" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="358" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A358" s="2">
+        <v>46122.333804988426</v>
+      </c>
+      <c r="B358" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C358" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D358" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E358" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F358" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G358" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="359" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A359" s="4">
+        <v>46122.33420369213</v>
+      </c>
+      <c r="B359" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C359" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D359" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E359" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F359" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G359" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="360" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A360" s="2">
+        <v>46122.33439001157</v>
+      </c>
+      <c r="B360" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C360" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D360" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E360" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F360" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G360" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="361" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A361" s="4">
+        <v>46122.37132832176</v>
+      </c>
+      <c r="B361" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C361" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D361" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E361" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F361" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G361" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="362" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A362" s="2">
+        <v>46122.450610995365</v>
+      </c>
+      <c r="B362" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C362" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D362" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E362" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F362" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G362" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="363" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A363" s="4">
+        <v>46122.51600920139</v>
+      </c>
+      <c r="B363" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C363" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D363" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E363" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F363" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G363" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="364" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A364" s="2">
+        <v>46123.18444614584</v>
+      </c>
+      <c r="B364" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C364" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D364" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E364" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F364" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G364" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="365" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A365" s="4">
+        <v>46123.18465393518</v>
+      </c>
+      <c r="B365" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C365" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D365" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E365" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F365" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G365" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="366" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A366" s="2">
+        <v>46123.19019862269</v>
+      </c>
+      <c r="B366" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C366" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D366" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E366" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F366" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G366" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="367" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A367" s="4">
+        <v>46123.192055798616</v>
+      </c>
+      <c r="B367" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C367" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D367" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E367" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F367" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="G367" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="368" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A368" s="2">
+        <v>46123.20587709491</v>
+      </c>
+      <c r="B368" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C368" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D368" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E368" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F368" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G368" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="369" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A369" s="4">
+        <v>46123.20725478009</v>
+      </c>
+      <c r="B369" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C369" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D369" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E369" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F369" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G369" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="370" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A370" s="2">
+        <v>46123.212663900464</v>
+      </c>
+      <c r="B370" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C370" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D370" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E370" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F370" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G370" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="371" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A371" s="4">
+        <v>46123.21316935185</v>
+      </c>
+      <c r="B371" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C371" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D371" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E371" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F371" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G371" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="372" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A372" s="2">
+        <v>46123.21853168981</v>
+      </c>
+      <c r="B372" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C372" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D372" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E372" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F372" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G372" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="373" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A373" s="4">
+        <v>46123.21928754629</v>
+      </c>
+      <c r="B373" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C373" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D373" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E373" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F373" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="G373" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="374" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A374" s="2">
+        <v>46123.220265254626</v>
+      </c>
+      <c r="B374" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C374" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D374" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E374" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F374" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="G374" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="375" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A375" s="4">
+        <v>46123.23323989584</v>
+      </c>
+      <c r="B375" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C375" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D375" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E375" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F375" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G375" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="376" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A376" s="2">
+        <v>46123.28142025463</v>
+      </c>
+      <c r="B376" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C376" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D376" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E376" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F376" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G376" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="377" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A377" s="4">
+        <v>46123.28978796296</v>
+      </c>
+      <c r="B377" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C377" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D377" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="E377" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F377" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G377" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="378" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A378" s="2">
+        <v>46123.29025873843</v>
+      </c>
+      <c r="B378" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C378" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D378" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E378" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F378" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G378" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="379" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A379" s="4">
+        <v>46123.29061391204</v>
+      </c>
+      <c r="B379" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C379" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D379" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E379" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F379" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G379" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="380" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A380" s="2">
+        <v>46123.29065047453</v>
+      </c>
+      <c r="B380" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C380" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D380" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E380" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F380" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="G380" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="381" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A381" s="4">
+        <v>46123.29094961805</v>
+      </c>
+      <c r="B381" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C381" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D381" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="E381" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F381" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G381" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="382" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A382" s="2">
+        <v>46123.292742314814</v>
+      </c>
+      <c r="B382" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C382" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D382" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E382" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F382" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G382" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="383" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A383" s="4">
+        <v>46123.29274600695</v>
+      </c>
+      <c r="B383" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C383" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D383" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="E383" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F383" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G383" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="384" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A384" s="2">
+        <v>46123.29439170139</v>
+      </c>
+      <c r="B384" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C384" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D384" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E384" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F384" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G384" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="385" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A385" s="4">
+        <v>46123.29638990741</v>
+      </c>
+      <c r="B385" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C385" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D385" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="E385" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F385" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G385" s="5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="386" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A386" s="2">
+        <v>46123.29712994213</v>
+      </c>
+      <c r="B386" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C386" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D386" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E386" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F386" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G386" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="387" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A387" s="4">
+        <v>46123.3241491088</v>
+      </c>
+      <c r="B387" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C387" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D387" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="E387" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F387" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G387" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="388" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A388" s="2">
+        <v>46123.32727443287</v>
+      </c>
+      <c r="B388" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C388" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D388" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E388" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F388" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G388" s="3" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="389" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A389" s="4">
+        <v>46155.2809508912</v>
+      </c>
+      <c r="B389" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C389" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D389" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="E389" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F389" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G389" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="390" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A390" s="2">
+        <v>46155.43479417824</v>
+      </c>
+      <c r="B390" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C390" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D390" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E390" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F390" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G390" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="391" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A391" s="4">
+        <v>46155.44487983796</v>
+      </c>
+      <c r="B391" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C391" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D391" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E391" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F391" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G391" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="392" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A392" s="2">
+        <v>46155.44516020833</v>
+      </c>
+      <c r="B392" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C392" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D392" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E392" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F392" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G392" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="393" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A393" s="4">
+        <v>46155.44526929398</v>
+      </c>
+      <c r="B393" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C393" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D393" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E393" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F393" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G393" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="394" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A394" s="2">
+        <v>46155.44543678241</v>
+      </c>
+      <c r="B394" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C394" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D394" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E394" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F394" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G394" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="395" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A395" s="4">
+        <v>46156.38913877315</v>
+      </c>
+      <c r="B395" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C395" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D395" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="E395" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F395" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G395" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="396" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A396" s="2">
+        <v>46156.393872326385</v>
+      </c>
+      <c r="B396" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C396" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D396" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E396" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F396" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G396" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="397" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A397" s="4">
+        <v>46156.394066608795</v>
+      </c>
+      <c r="B397" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C397" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D397" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="E397" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F397" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G397" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="398" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A398" s="2">
+        <v>46158.23980258102</v>
+      </c>
+      <c r="B398" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C398" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D398" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="E398" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F398" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G398" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="399" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A399" s="4">
+        <v>46158.240449097226</v>
+      </c>
+      <c r="B399" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C399" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D399" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="E399" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F399" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G399" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="400" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A400" s="2">
+        <v>46158.24170141204</v>
+      </c>
+      <c r="B400" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C400" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D400" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E400" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F400" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G400" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="401" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A401" s="4">
+        <v>46158.2418666088</v>
+      </c>
+      <c r="B401" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C401" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D401" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E401" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F401" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G401" s="5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="402" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A402" s="2">
+        <v>46158.241902546295</v>
+      </c>
+      <c r="B402" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C402" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D402" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E402" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F402" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G402" s="3" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="403" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A403" s="4">
+        <v>46158.24230780093</v>
+      </c>
+      <c r="B403" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C403" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D403" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="E403" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F403" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G403" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="404" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A404" s="2">
+        <v>46158.24234140046</v>
+      </c>
+      <c r="B404" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C404" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D404" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="E404" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F404" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G404" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="405" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A405" s="4">
+        <v>46158.24867403935</v>
+      </c>
+      <c r="B405" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C405" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D405" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E405" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F405" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G405" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="406" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A406" s="2">
+        <v>46158.248676030096</v>
+      </c>
+      <c r="B406" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C406" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D406" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E406" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F406" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G406" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="407" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A407" s="4">
+        <v>46158.24868798611</v>
+      </c>
+      <c r="B407" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C407" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D407" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E407" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F407" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G407" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="408" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A408" s="2">
+        <v>46158.24870034722</v>
+      </c>
+      <c r="B408" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C408" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D408" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E408" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F408" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G408" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="409" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A409" s="4">
+        <v>46158.249244363426</v>
+      </c>
+      <c r="B409" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C409" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D409" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E409" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F409" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G409" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="410" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A410" s="2">
+        <v>46158.249249942135</v>
+      </c>
+      <c r="B410" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C410" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D410" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E410" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F410" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G410" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="411" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A411" s="4">
+        <v>46158.24925607639</v>
+      </c>
+      <c r="B411" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C411" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D411" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E411" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F411" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G411" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="412" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A412" s="2">
+        <v>46158.24926216435</v>
+      </c>
+      <c r="B412" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C412" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D412" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E412" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F412" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G412" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="413" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A413" s="4">
+        <v>46158.24927118055</v>
+      </c>
+      <c r="B413" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C413" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D413" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E413" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F413" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G413" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="414" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A414" s="2">
+        <v>46158.249279131946</v>
+      </c>
+      <c r="B414" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C414" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D414" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E414" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F414" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G414" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="415" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A415" s="4">
+        <v>46158.24929310185</v>
+      </c>
+      <c r="B415" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C415" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D415" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E415" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F415" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G415" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="416" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A416" s="2">
+        <v>46158.24930114583</v>
+      </c>
+      <c r="B416" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C416" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D416" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E416" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F416" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G416" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="417" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A417" s="4">
+        <v>46158.26074149305</v>
+      </c>
+      <c r="B417" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C417" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D417" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="E417" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F417" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G417" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="418" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A418" s="2">
+        <v>46158.260746608794</v>
+      </c>
+      <c r="B418" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C418" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D418" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="E418" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F418" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G418" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="419" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A419" s="4">
+        <v>46158.271334247685</v>
+      </c>
+      <c r="B419" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C419" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D419" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E419" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F419" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G419" s="5" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="420" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A420" s="2">
+        <v>46158.27678487268</v>
+      </c>
+      <c r="B420" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C420" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D420" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="E420" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F420" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G420" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="421" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A421" s="4">
+        <v>46158.27679319444</v>
+      </c>
+      <c r="B421" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C421" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D421" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E421" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F421" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G421" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="422" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A422" s="2">
+        <v>46158.30981542824</v>
+      </c>
+      <c r="B422" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C422" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D422" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E422" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F422" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G422" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="423" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A423" s="4">
+        <v>46158.31039699074</v>
+      </c>
+      <c r="B423" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C423" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D423" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E423" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F423" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G423" s="5" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="424" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A424" s="2">
+        <v>46195.482533055554</v>
+      </c>
+      <c r="B424" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C424" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D424" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E424" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F424" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G424" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>